<commit_message>
Panel administrador Obito con ranking y faltantes
</commit_message>
<xml_diff>
--- a/miembros1.xlsx
+++ b/miembros1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Sistemascomites\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5189F86B-D85C-4880-AE70-C5E848CEDD4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22F78B61-B215-4D2F-A228-A45C9EA87F91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{4388099F-EC29-4ACA-BFE4-DD6000085508}"/>
   </bookViews>
@@ -78,9 +78,6 @@
     <t>Alex Ryutakeshi Cazorla Abanto</t>
   </si>
   <si>
-    <t>Gian Franco Altamirano Torres</t>
-  </si>
-  <si>
     <t>Xavier Fidel Dueñas Sixto</t>
   </si>
   <si>
@@ -556,6 +553,9 @@
   </si>
   <si>
     <t xml:space="preserve">Juan Angel Bustamante Vasquez </t>
+  </si>
+  <si>
+    <t>Gian Franco Altamirano Torres 🌀</t>
   </si>
 </sst>
 </file>
@@ -1015,7 +1015,7 @@
   <dimension ref="A1:I333"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="39.33203125" customWidth="1"/>
+    <col min="1" max="1" width="43" customWidth="1"/>
     <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25.6640625" customWidth="1"/>
@@ -1027,7 +1027,7 @@
         <v>1</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>2</v>
@@ -1049,7 +1049,7 @@
         <v>946396819</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E2" s="5"/>
       <c r="F2" s="4"/>
@@ -1065,7 +1065,7 @@
         <v>948450774</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E3" s="5"/>
       <c r="F3" s="4"/>
@@ -1081,7 +1081,7 @@
         <v>960668392</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E4" s="5"/>
       <c r="F4" s="4"/>
@@ -1097,7 +1097,7 @@
         <v>983499728</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E5" s="5"/>
       <c r="F5" s="4"/>
@@ -1113,7 +1113,7 @@
         <v>948164104</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="4"/>
@@ -1129,7 +1129,7 @@
         <v>978414015</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E7" s="5"/>
       <c r="F7" s="4"/>
@@ -1145,7 +1145,7 @@
         <v>974320645</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E8" s="5"/>
       <c r="F8" s="4"/>
@@ -1161,7 +1161,7 @@
         <v>931218653</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E9" s="5"/>
       <c r="F9" s="4"/>
@@ -1177,7 +1177,7 @@
         <v>993861268</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E10" s="5"/>
       <c r="F10" s="4"/>
@@ -1193,16 +1193,16 @@
         <v>912097319</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E11" s="5"/>
       <c r="F11" s="4"/>
       <c r="G11" s="5"/>
       <c r="I11" s="1"/>
     </row>
-    <row r="12" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="14" t="s">
-        <v>13</v>
+        <v>172</v>
       </c>
       <c r="B12" s="14">
         <v>75406534</v>
@@ -1211,7 +1211,7 @@
         <v>916914496</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E12" s="5"/>
       <c r="F12" s="4"/>
@@ -1220,14 +1220,14 @@
     </row>
     <row r="13" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" s="14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13" s="14"/>
       <c r="C13" s="14">
         <v>949360902</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E13" s="5"/>
       <c r="F13" s="4"/>
@@ -1236,14 +1236,14 @@
     </row>
     <row r="14" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B14" s="14"/>
       <c r="C14" s="14">
         <v>942377823</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E14" s="5"/>
       <c r="F14" s="4"/>
@@ -1252,14 +1252,14 @@
     </row>
     <row r="15" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B15" s="14"/>
       <c r="C15" s="14">
         <v>945247890</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E15" s="5"/>
       <c r="F15" s="4"/>
@@ -1268,14 +1268,14 @@
     </row>
     <row r="16" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B16" s="14"/>
       <c r="C16" s="14">
         <v>930768232</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E16" s="5"/>
       <c r="F16" s="4"/>
@@ -1284,14 +1284,14 @@
     </row>
     <row r="17" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" s="14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B17" s="14"/>
       <c r="C17" s="14">
         <v>959358156</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E17" s="5"/>
       <c r="F17" s="4"/>
@@ -1300,14 +1300,14 @@
     </row>
     <row r="18" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B18" s="14"/>
       <c r="C18" s="14">
         <v>934497322</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E18" s="5"/>
       <c r="F18" s="4"/>
@@ -1316,14 +1316,14 @@
     </row>
     <row r="19" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" s="14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B19" s="14"/>
       <c r="C19" s="14">
         <v>979389805</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E19" s="5"/>
       <c r="F19" s="4"/>
@@ -1332,14 +1332,14 @@
     </row>
     <row r="20" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B20" s="14"/>
       <c r="C20" s="14">
         <v>942240935</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E20" s="5"/>
       <c r="F20" s="4"/>
@@ -1348,14 +1348,14 @@
     </row>
     <row r="21" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B21" s="14"/>
       <c r="C21" s="14">
         <v>945974523</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E21" s="5"/>
       <c r="F21" s="4"/>
@@ -1364,14 +1364,14 @@
     </row>
     <row r="22" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B22" s="14"/>
       <c r="C22" s="14">
         <v>940348698</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E22" s="5"/>
       <c r="F22" s="4"/>
@@ -1380,14 +1380,14 @@
     </row>
     <row r="23" spans="1:9" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B23" s="14"/>
       <c r="C23" s="14">
         <v>972627155</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E23" s="5"/>
       <c r="F23" s="4"/>
@@ -1396,14 +1396,14 @@
     </row>
     <row r="24" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B24" s="14"/>
       <c r="C24" s="14">
         <v>989086745</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E24" s="5"/>
       <c r="F24" s="4"/>
@@ -1412,14 +1412,14 @@
     </row>
     <row r="25" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B25" s="14"/>
       <c r="C25" s="14">
         <v>912578553</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E25" s="5"/>
       <c r="F25" s="4"/>
@@ -1428,14 +1428,14 @@
     </row>
     <row r="26" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="14" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B26" s="14"/>
       <c r="C26" s="14">
         <v>900605129</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E26" s="5"/>
       <c r="F26" s="4"/>
@@ -1444,14 +1444,14 @@
     </row>
     <row r="27" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" s="14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B27" s="14"/>
       <c r="C27" s="14">
         <v>906571483</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E27" s="5"/>
       <c r="F27" s="4"/>
@@ -1460,14 +1460,14 @@
     </row>
     <row r="28" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B28" s="14"/>
       <c r="C28" s="14">
         <v>912578553</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E28" s="5"/>
       <c r="F28" s="4"/>
@@ -1476,14 +1476,14 @@
     </row>
     <row r="29" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A29" s="14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B29" s="14"/>
       <c r="C29" s="14">
         <v>964767294</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E29" s="5"/>
       <c r="F29" s="4"/>
@@ -1492,14 +1492,14 @@
     </row>
     <row r="30" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B30" s="14"/>
       <c r="C30" s="14">
         <v>970129002</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E30" s="5"/>
       <c r="F30" s="4"/>
@@ -1508,14 +1508,14 @@
     </row>
     <row r="31" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A31" s="14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B31" s="14"/>
       <c r="C31" s="14">
         <v>935447293</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E31" s="5"/>
       <c r="F31" s="4"/>
@@ -1524,14 +1524,14 @@
     </row>
     <row r="32" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B32" s="14"/>
       <c r="C32" s="14">
         <v>930359429</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E32" s="5"/>
       <c r="F32" s="4"/>
@@ -1540,14 +1540,14 @@
     </row>
     <row r="33" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A33" s="14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B33" s="14"/>
       <c r="C33" s="14">
         <v>947148712</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E33" s="5"/>
       <c r="F33" s="4"/>
@@ -1556,14 +1556,14 @@
     </row>
     <row r="34" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B34" s="14"/>
       <c r="C34" s="14">
         <v>917129115</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E34" s="5"/>
       <c r="F34" s="4"/>
@@ -1572,14 +1572,14 @@
     </row>
     <row r="35" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A35" s="14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B35" s="14"/>
       <c r="C35" s="14">
         <v>938175835</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E35" s="5"/>
       <c r="F35" s="4"/>
@@ -1588,14 +1588,14 @@
     </row>
     <row r="36" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B36" s="14"/>
       <c r="C36" s="14">
         <v>992848081</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E36" s="5"/>
       <c r="F36" s="4"/>
@@ -1604,14 +1604,14 @@
     </row>
     <row r="37" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A37" s="14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B37" s="14"/>
       <c r="C37" s="14">
         <v>968886681</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E37" s="5"/>
       <c r="F37" s="4"/>
@@ -1620,14 +1620,14 @@
     </row>
     <row r="38" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B38" s="14"/>
       <c r="C38" s="14">
         <v>963657042</v>
       </c>
       <c r="D38" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E38" s="5"/>
       <c r="F38" s="4"/>
@@ -1636,14 +1636,14 @@
     </row>
     <row r="39" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A39" s="14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B39" s="14"/>
       <c r="C39" s="14">
         <v>924509788</v>
       </c>
       <c r="D39" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E39" s="5"/>
       <c r="F39" s="4"/>
@@ -1652,14 +1652,14 @@
     </row>
     <row r="40" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B40" s="14"/>
       <c r="C40" s="14">
         <v>944019208</v>
       </c>
       <c r="D40" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E40" s="5"/>
       <c r="F40" s="4"/>
@@ -1668,14 +1668,14 @@
     </row>
     <row r="41" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A41" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B41" s="14"/>
       <c r="C41" s="14">
         <v>993336109</v>
       </c>
       <c r="D41" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E41" s="5"/>
       <c r="F41" s="4"/>
@@ -1684,14 +1684,14 @@
     </row>
     <row r="42" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B42" s="14"/>
       <c r="C42" s="14">
         <v>959454929</v>
       </c>
       <c r="D42" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E42" s="5"/>
       <c r="F42" s="4"/>
@@ -1700,14 +1700,14 @@
     </row>
     <row r="43" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A43" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B43" s="14"/>
       <c r="C43" s="14">
         <v>919195204</v>
       </c>
       <c r="D43" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E43" s="5"/>
       <c r="F43" s="4"/>
@@ -1716,14 +1716,14 @@
     </row>
     <row r="44" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B44" s="14"/>
       <c r="C44" s="14">
         <v>902049993</v>
       </c>
       <c r="D44" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E44" s="5"/>
       <c r="F44" s="4"/>
@@ -1732,14 +1732,14 @@
     </row>
     <row r="45" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B45" s="14"/>
       <c r="C45" s="14">
         <v>981379273</v>
       </c>
       <c r="D45" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E45" s="5"/>
       <c r="F45" s="4"/>
@@ -1748,14 +1748,14 @@
     </row>
     <row r="46" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B46" s="14"/>
       <c r="C46" s="14">
         <v>993336109</v>
       </c>
       <c r="D46" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E46" s="5"/>
       <c r="F46" s="4"/>
@@ -1764,14 +1764,14 @@
     </row>
     <row r="47" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A47" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B47" s="14"/>
       <c r="C47" s="14">
         <v>910120852</v>
       </c>
       <c r="D47" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E47" s="5"/>
       <c r="F47" s="4"/>
@@ -1780,14 +1780,14 @@
     </row>
     <row r="48" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B48" s="14"/>
       <c r="C48" s="14">
         <v>962201027</v>
       </c>
       <c r="D48" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E48" s="5"/>
       <c r="F48" s="4"/>
@@ -1796,14 +1796,14 @@
     </row>
     <row r="49" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A49" s="14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B49" s="14"/>
       <c r="C49" s="14">
         <v>977523229</v>
       </c>
       <c r="D49" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E49" s="5"/>
       <c r="F49" s="4"/>
@@ -1812,14 +1812,14 @@
     </row>
     <row r="50" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="14" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B50" s="14"/>
       <c r="C50" s="14">
         <v>978956780</v>
       </c>
       <c r="D50" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E50" s="5"/>
       <c r="F50" s="4"/>
@@ -1828,14 +1828,14 @@
     </row>
     <row r="51" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A51" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B51" s="14"/>
       <c r="C51" s="14">
         <v>967462521</v>
       </c>
       <c r="D51" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E51" s="5"/>
       <c r="F51" s="4"/>
@@ -1844,14 +1844,14 @@
     </row>
     <row r="52" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B52" s="14"/>
       <c r="C52" s="14">
         <v>986957330</v>
       </c>
       <c r="D52" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E52" s="5"/>
       <c r="F52" s="4"/>
@@ -1860,14 +1860,14 @@
     </row>
     <row r="53" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A53" s="14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B53" s="14"/>
       <c r="C53" s="14">
         <v>968226851</v>
       </c>
       <c r="D53" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E53" s="5"/>
       <c r="F53" s="4"/>
@@ -1876,14 +1876,14 @@
     </row>
     <row r="54" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B54" s="14"/>
       <c r="C54" s="14">
         <v>921990078</v>
       </c>
       <c r="D54" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E54" s="5"/>
       <c r="F54" s="4"/>
@@ -1892,14 +1892,14 @@
     </row>
     <row r="55" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A55" s="14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B55" s="14"/>
       <c r="C55" s="14">
         <v>917221161</v>
       </c>
       <c r="D55" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E55" s="5"/>
       <c r="F55" s="4"/>
@@ -1908,14 +1908,14 @@
     </row>
     <row r="56" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B56" s="14"/>
       <c r="C56" s="14">
         <v>974848826</v>
       </c>
       <c r="D56" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E56" s="5"/>
       <c r="F56" s="4"/>
@@ -1924,14 +1924,14 @@
     </row>
     <row r="57" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A57" s="14" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B57" s="14"/>
       <c r="C57" s="14">
         <v>938884360</v>
       </c>
       <c r="D57" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E57" s="5"/>
       <c r="F57" s="4"/>
@@ -1940,14 +1940,14 @@
     </row>
     <row r="58" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="14" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B58" s="14"/>
       <c r="C58" s="14">
         <v>963589472</v>
       </c>
       <c r="D58" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E58" s="5"/>
       <c r="F58" s="4"/>
@@ -1956,14 +1956,14 @@
     </row>
     <row r="59" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A59" s="14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B59" s="14"/>
       <c r="C59" s="14">
         <v>984937208</v>
       </c>
       <c r="D59" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E59" s="5"/>
       <c r="F59" s="4"/>
@@ -1972,14 +1972,14 @@
     </row>
     <row r="60" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B60" s="14"/>
       <c r="C60" s="14">
         <v>916281061</v>
       </c>
       <c r="D60" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E60" s="5"/>
       <c r="F60" s="4"/>
@@ -1988,14 +1988,14 @@
     </row>
     <row r="61" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A61" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B61" s="14"/>
       <c r="C61" s="14">
         <v>931774461</v>
       </c>
       <c r="D61" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E61" s="5"/>
       <c r="F61" s="4"/>
@@ -2004,14 +2004,14 @@
     </row>
     <row r="62" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B62" s="14"/>
       <c r="C62" s="14">
         <v>927679081</v>
       </c>
       <c r="D62" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E62" s="5"/>
       <c r="F62" s="4"/>
@@ -2020,14 +2020,14 @@
     </row>
     <row r="63" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A63" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B63" s="14"/>
       <c r="C63" s="14">
         <v>932630425</v>
       </c>
       <c r="D63" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E63" s="5"/>
       <c r="F63" s="4"/>
@@ -2036,14 +2036,14 @@
     </row>
     <row r="64" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="14" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B64" s="14"/>
       <c r="C64" s="14">
         <v>900539013</v>
       </c>
       <c r="D64" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E64" s="5"/>
       <c r="F64" s="4"/>
@@ -2052,14 +2052,14 @@
     </row>
     <row r="65" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A65" s="14" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B65" s="14"/>
       <c r="C65" s="14">
         <v>919677598</v>
       </c>
       <c r="D65" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E65" s="5"/>
       <c r="F65" s="4"/>
@@ -2068,14 +2068,14 @@
     </row>
     <row r="66" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B66" s="14"/>
       <c r="C66" s="14">
         <v>994321341</v>
       </c>
       <c r="D66" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E66" s="5"/>
       <c r="F66" s="4"/>
@@ -2084,14 +2084,14 @@
     </row>
     <row r="67" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A67" s="14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B67" s="14"/>
       <c r="C67" s="14">
         <v>940859311</v>
       </c>
       <c r="D67" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E67" s="5"/>
       <c r="F67" s="4"/>
@@ -2100,14 +2100,14 @@
     </row>
     <row r="68" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B68" s="14"/>
       <c r="C68" s="14">
         <v>987124440</v>
       </c>
       <c r="D68" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E68" s="5"/>
       <c r="F68" s="4"/>
@@ -2116,14 +2116,14 @@
     </row>
     <row r="69" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A69" s="14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B69" s="14"/>
       <c r="C69" s="14">
         <v>977576131</v>
       </c>
       <c r="D69" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E69" s="5"/>
       <c r="F69" s="4"/>
@@ -2132,14 +2132,14 @@
     </row>
     <row r="70" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B70" s="14"/>
       <c r="C70" s="14">
         <v>950324370</v>
       </c>
       <c r="D70" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E70" s="5"/>
       <c r="F70" s="4"/>
@@ -2148,14 +2148,14 @@
     </row>
     <row r="71" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A71" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B71" s="14"/>
       <c r="C71" s="14">
         <v>924797687</v>
       </c>
       <c r="D71" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E71" s="5"/>
       <c r="F71" s="4"/>
@@ -2164,14 +2164,14 @@
     </row>
     <row r="72" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B72" s="14"/>
       <c r="C72" s="14">
         <v>904931317</v>
       </c>
       <c r="D72" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E72" s="5"/>
       <c r="F72" s="4"/>
@@ -2180,14 +2180,14 @@
     </row>
     <row r="73" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A73" s="14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B73" s="14"/>
       <c r="C73" s="14">
         <v>990026654</v>
       </c>
       <c r="D73" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E73" s="5"/>
       <c r="F73" s="4"/>
@@ -2196,14 +2196,14 @@
     </row>
     <row r="74" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B74" s="14"/>
       <c r="C74" s="14">
         <v>952965327</v>
       </c>
       <c r="D74" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E74" s="5"/>
       <c r="F74" s="4"/>
@@ -2212,14 +2212,14 @@
     </row>
     <row r="75" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A75" s="14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B75" s="14"/>
       <c r="C75" s="14">
         <v>989918323</v>
       </c>
       <c r="D75" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E75" s="5"/>
       <c r="F75" s="4"/>
@@ -2228,14 +2228,14 @@
     </row>
     <row r="76" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="14" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B76" s="14"/>
       <c r="C76" s="14">
         <v>946738790</v>
       </c>
       <c r="D76" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E76" s="5"/>
       <c r="F76" s="4"/>
@@ -2244,14 +2244,14 @@
     </row>
     <row r="77" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A77" s="14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B77" s="14"/>
       <c r="C77" s="14">
         <v>922351225</v>
       </c>
       <c r="D77" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E77" s="5"/>
       <c r="F77" s="4"/>
@@ -2260,14 +2260,14 @@
     </row>
     <row r="78" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B78" s="14"/>
       <c r="C78" s="14">
         <v>929511047</v>
       </c>
       <c r="D78" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E78" s="5"/>
       <c r="F78" s="4"/>
@@ -2276,14 +2276,14 @@
     </row>
     <row r="79" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A79" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B79" s="14"/>
       <c r="C79" s="14">
         <v>979556426</v>
       </c>
       <c r="D79" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E79" s="5"/>
       <c r="F79" s="4"/>
@@ -2292,14 +2292,14 @@
     </row>
     <row r="80" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B80" s="14"/>
       <c r="C80" s="14">
         <v>940453146</v>
       </c>
       <c r="D80" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E80" s="5"/>
       <c r="F80" s="4"/>
@@ -2308,14 +2308,14 @@
     </row>
     <row r="81" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A81" s="14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B81" s="14"/>
       <c r="C81" s="14">
         <v>993141165</v>
       </c>
       <c r="D81" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E81" s="5"/>
       <c r="F81" s="4"/>
@@ -2324,14 +2324,14 @@
     </row>
     <row r="82" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B82" s="14"/>
       <c r="C82" s="14">
         <v>965254714</v>
       </c>
       <c r="D82" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E82" s="5"/>
       <c r="F82" s="4"/>
@@ -2340,14 +2340,14 @@
     </row>
     <row r="83" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A83" s="14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B83" s="14"/>
       <c r="C83" s="14">
         <v>986267014</v>
       </c>
       <c r="D83" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E83" s="5"/>
       <c r="F83" s="4"/>
@@ -2356,14 +2356,14 @@
     </row>
     <row r="84" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B84" s="14"/>
       <c r="C84" s="14">
         <v>926948069</v>
       </c>
       <c r="D84" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E84" s="5"/>
       <c r="F84" s="4"/>
@@ -2372,14 +2372,14 @@
     </row>
     <row r="85" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A85" s="14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B85" s="14"/>
       <c r="C85" s="14">
         <v>987010169</v>
       </c>
       <c r="D85" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E85" s="5"/>
       <c r="F85" s="4"/>
@@ -2388,14 +2388,14 @@
     </row>
     <row r="86" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B86" s="14"/>
       <c r="C86" s="14">
         <v>980692014</v>
       </c>
       <c r="D86" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E86" s="5"/>
       <c r="F86" s="4"/>
@@ -2404,14 +2404,14 @@
     </row>
     <row r="87" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A87" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B87" s="14"/>
       <c r="C87" s="14">
         <v>939925601</v>
       </c>
       <c r="D87" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E87" s="5"/>
       <c r="F87" s="4"/>
@@ -2420,14 +2420,14 @@
     </row>
     <row r="88" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B88" s="14"/>
       <c r="C88" s="14">
         <v>949222202</v>
       </c>
       <c r="D88" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E88" s="5"/>
       <c r="F88" s="4"/>
@@ -2436,14 +2436,14 @@
     </row>
     <row r="89" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A89" s="14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B89" s="14"/>
       <c r="C89" s="14">
         <v>953116755</v>
       </c>
       <c r="D89" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E89" s="5"/>
       <c r="F89" s="4"/>
@@ -2452,14 +2452,14 @@
     </row>
     <row r="90" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B90" s="14"/>
       <c r="C90" s="14">
         <v>984022907</v>
       </c>
       <c r="D90" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E90" s="5"/>
       <c r="F90" s="4"/>
@@ -2468,14 +2468,14 @@
     </row>
     <row r="91" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A91" s="14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B91" s="14"/>
       <c r="C91" s="14">
         <v>940661131</v>
       </c>
       <c r="D91" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E91" s="5"/>
       <c r="F91" s="4"/>
@@ -2484,14 +2484,14 @@
     </row>
     <row r="92" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="14" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B92" s="14"/>
       <c r="C92" s="14">
         <v>991829531</v>
       </c>
       <c r="D92" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E92" s="5"/>
       <c r="F92" s="4"/>
@@ -2500,14 +2500,14 @@
     </row>
     <row r="93" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A93" s="14" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B93" s="14"/>
       <c r="C93" s="14">
         <v>984877034</v>
       </c>
       <c r="D93" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E93" s="5"/>
       <c r="F93" s="4"/>
@@ -2516,14 +2516,14 @@
     </row>
     <row r="94" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="14" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B94" s="14"/>
       <c r="C94" s="14">
         <v>968185040</v>
       </c>
       <c r="D94" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E94" s="5"/>
       <c r="F94" s="4"/>
@@ -2532,14 +2532,14 @@
     </row>
     <row r="95" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A95" s="14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B95" s="14"/>
       <c r="C95" s="14">
         <v>949700807</v>
       </c>
       <c r="D95" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E95" s="5"/>
       <c r="F95" s="4"/>
@@ -2548,14 +2548,14 @@
     </row>
     <row r="96" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="14" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B96" s="14"/>
       <c r="C96" s="14">
         <v>980322820</v>
       </c>
       <c r="D96" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E96" s="5"/>
       <c r="F96" s="4"/>
@@ -2564,14 +2564,14 @@
     </row>
     <row r="97" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A97" s="14" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B97" s="14"/>
       <c r="C97" s="14">
         <v>974178840</v>
       </c>
       <c r="D97" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E97" s="5"/>
       <c r="F97" s="4"/>
@@ -2580,14 +2580,14 @@
     </row>
     <row r="98" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B98" s="14"/>
       <c r="C98" s="14">
         <v>938872455</v>
       </c>
       <c r="D98" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E98" s="5"/>
       <c r="F98" s="4"/>
@@ -2596,14 +2596,14 @@
     </row>
     <row r="99" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A99" s="14" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B99" s="14"/>
       <c r="C99" s="14">
         <v>900148108</v>
       </c>
       <c r="D99" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E99" s="5"/>
       <c r="F99" s="4"/>
@@ -2612,14 +2612,14 @@
     </row>
     <row r="100" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B100" s="14"/>
       <c r="C100" s="14">
         <v>997000215</v>
       </c>
       <c r="D100" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E100" s="5"/>
       <c r="F100" s="4"/>
@@ -2628,14 +2628,14 @@
     </row>
     <row r="101" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A101" s="14" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B101" s="14"/>
       <c r="C101" s="14">
         <v>975665973</v>
       </c>
       <c r="D101" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E101" s="5"/>
       <c r="F101" s="4"/>
@@ -2644,14 +2644,14 @@
     </row>
     <row r="102" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B102" s="14"/>
       <c r="C102" s="14">
         <v>926879719</v>
       </c>
       <c r="D102" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E102" s="5"/>
       <c r="F102" s="4"/>
@@ -2660,14 +2660,14 @@
     </row>
     <row r="103" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A103" s="14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B103" s="14"/>
       <c r="C103" s="14">
         <v>950954215</v>
       </c>
       <c r="D103" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E103" s="5"/>
       <c r="F103" s="4"/>
@@ -2676,14 +2676,14 @@
     </row>
     <row r="104" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B104" s="14"/>
       <c r="C104" s="14">
         <v>994409997</v>
       </c>
       <c r="D104" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E104" s="5"/>
       <c r="F104" s="4"/>
@@ -2692,14 +2692,14 @@
     </row>
     <row r="105" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A105" s="14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B105" s="14"/>
       <c r="C105" s="14">
         <v>994144910</v>
       </c>
       <c r="D105" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E105" s="5"/>
       <c r="F105" s="4"/>
@@ -2708,14 +2708,14 @@
     </row>
     <row r="106" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B106" s="14"/>
       <c r="C106" s="14">
         <v>918975279</v>
       </c>
       <c r="D106" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E106" s="5"/>
       <c r="F106" s="4"/>
@@ -2724,14 +2724,14 @@
     </row>
     <row r="107" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A107" s="14" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B107" s="14"/>
       <c r="C107" s="14">
         <v>952616806</v>
       </c>
       <c r="D107" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E107" s="5"/>
       <c r="F107" s="4"/>
@@ -2740,14 +2740,14 @@
     </row>
     <row r="108" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="14" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B108" s="14"/>
       <c r="C108" s="14">
         <v>977742714</v>
       </c>
       <c r="D108" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E108" s="5"/>
       <c r="F108" s="4"/>
@@ -2756,14 +2756,14 @@
     </row>
     <row r="109" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A109" s="14" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B109" s="14"/>
       <c r="C109" s="14">
         <v>980542461</v>
       </c>
       <c r="D109" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E109" s="5"/>
       <c r="F109" s="4"/>
@@ -2772,14 +2772,14 @@
     </row>
     <row r="110" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="14" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B110" s="14"/>
       <c r="C110" s="14">
         <v>904445866</v>
       </c>
       <c r="D110" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E110" s="5"/>
       <c r="F110" s="4"/>
@@ -2788,14 +2788,14 @@
     </row>
     <row r="111" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A111" s="14" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B111" s="14"/>
       <c r="C111" s="14">
         <v>942580610</v>
       </c>
       <c r="D111" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E111" s="5"/>
       <c r="F111" s="4"/>
@@ -2804,14 +2804,14 @@
     </row>
     <row r="112" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="14" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B112" s="14"/>
       <c r="C112" s="14">
         <v>926119735</v>
       </c>
       <c r="D112" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E112" s="5"/>
       <c r="F112" s="4"/>
@@ -2820,14 +2820,14 @@
     </row>
     <row r="113" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A113" s="14" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B113" s="14"/>
       <c r="C113" s="14" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D113" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E113" s="5"/>
       <c r="F113" s="4"/>
@@ -2836,14 +2836,14 @@
     </row>
     <row r="114" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="14" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B114" s="14"/>
       <c r="C114" s="14">
         <v>913158865</v>
       </c>
       <c r="D114" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E114" s="5"/>
       <c r="F114" s="4"/>
@@ -2852,14 +2852,14 @@
     </row>
     <row r="115" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A115" s="14" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B115" s="14"/>
       <c r="C115" s="14">
         <v>933858695</v>
       </c>
       <c r="D115" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E115" s="5"/>
       <c r="F115" s="4"/>
@@ -2868,12 +2868,12 @@
     </row>
     <row r="116" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B116" s="14"/>
       <c r="C116" s="14"/>
       <c r="D116" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E116" s="5"/>
       <c r="F116" s="4"/>
@@ -2882,14 +2882,14 @@
     </row>
     <row r="117" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A117" s="14" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B117" s="14"/>
       <c r="C117" s="14">
         <v>933009187</v>
       </c>
       <c r="D117" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E117" s="5"/>
       <c r="F117" s="4"/>
@@ -2898,14 +2898,14 @@
     </row>
     <row r="118" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B118" s="14"/>
       <c r="C118" s="14">
         <v>949989617</v>
       </c>
       <c r="D118" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E118" s="5"/>
       <c r="F118" s="4"/>
@@ -2914,14 +2914,14 @@
     </row>
     <row r="119" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A119" s="14" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B119" s="14"/>
       <c r="C119" s="14">
         <v>917000180</v>
       </c>
       <c r="D119" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E119" s="5"/>
       <c r="F119" s="4"/>
@@ -2930,14 +2930,14 @@
     </row>
     <row r="120" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B120" s="14"/>
       <c r="C120" s="14">
         <v>949610154</v>
       </c>
       <c r="D120" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E120" s="5"/>
       <c r="F120" s="4"/>
@@ -2946,14 +2946,14 @@
     </row>
     <row r="121" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A121" s="14" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B121" s="14"/>
       <c r="C121" s="14">
         <v>933277756</v>
       </c>
       <c r="D121" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E121" s="5"/>
       <c r="F121" s="4"/>
@@ -2962,14 +2962,14 @@
     </row>
     <row r="122" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="14" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B122" s="14"/>
       <c r="C122" s="14">
         <v>972015817</v>
       </c>
       <c r="D122" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E122" s="5"/>
       <c r="F122" s="4"/>
@@ -2978,14 +2978,14 @@
     </row>
     <row r="123" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A123" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B123" s="14"/>
       <c r="C123" s="14">
         <v>925843970</v>
       </c>
       <c r="D123" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E123" s="5"/>
       <c r="F123" s="4"/>
@@ -2994,14 +2994,14 @@
     </row>
     <row r="124" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A124" s="14" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B124" s="14"/>
       <c r="C124" s="14">
         <v>928804324</v>
       </c>
       <c r="D124" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E124" s="5"/>
       <c r="F124" s="4"/>
@@ -3010,14 +3010,14 @@
     </row>
     <row r="125" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A125" s="14" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B125" s="14"/>
       <c r="C125" s="14">
         <v>902570315</v>
       </c>
       <c r="D125" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E125" s="5"/>
       <c r="F125" s="4"/>
@@ -3026,14 +3026,14 @@
     </row>
     <row r="126" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="14" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B126" s="14"/>
       <c r="C126" s="14">
         <v>916660021</v>
       </c>
       <c r="D126" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E126" s="5"/>
       <c r="F126" s="4"/>
@@ -3042,14 +3042,14 @@
     </row>
     <row r="127" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A127" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B127" s="14"/>
       <c r="C127" s="14">
         <v>900302292</v>
       </c>
       <c r="D127" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E127" s="5"/>
       <c r="F127" s="4"/>
@@ -3058,14 +3058,14 @@
     </row>
     <row r="128" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A128" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B128" s="14"/>
       <c r="C128" s="14">
         <v>931247256</v>
       </c>
       <c r="D128" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E128" s="5"/>
       <c r="F128" s="4"/>
@@ -3074,14 +3074,14 @@
     </row>
     <row r="129" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A129" s="14" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B129" s="14"/>
       <c r="C129" s="14">
         <v>950452975</v>
       </c>
       <c r="D129" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E129" s="5"/>
       <c r="F129" s="4"/>
@@ -3090,14 +3090,14 @@
     </row>
     <row r="130" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="14" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B130" s="14"/>
       <c r="C130" s="14">
         <v>947542469</v>
       </c>
       <c r="D130" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E130" s="5"/>
       <c r="F130" s="4"/>
@@ -3106,14 +3106,14 @@
     </row>
     <row r="131" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A131" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B131" s="14"/>
       <c r="C131" s="14">
         <v>908579375</v>
       </c>
       <c r="D131" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E131" s="5"/>
       <c r="F131" s="4"/>
@@ -3122,14 +3122,14 @@
     </row>
     <row r="132" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A132" s="14" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B132" s="14"/>
       <c r="C132" s="14">
         <v>907475286</v>
       </c>
       <c r="D132" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E132" s="5"/>
       <c r="F132" s="4"/>
@@ -3138,14 +3138,14 @@
     </row>
     <row r="133" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A133" s="14" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B133" s="14"/>
       <c r="C133" s="14">
         <v>994338876</v>
       </c>
       <c r="D133" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E133" s="5"/>
       <c r="F133" s="4"/>
@@ -3154,14 +3154,14 @@
     </row>
     <row r="134" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A134" s="14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B134" s="14"/>
       <c r="C134" s="14">
         <v>964839306</v>
       </c>
       <c r="D134" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E134" s="5"/>
       <c r="F134" s="4"/>
@@ -3170,14 +3170,14 @@
     </row>
     <row r="135" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A135" s="14" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B135" s="14"/>
       <c r="C135" s="14">
         <v>913536643</v>
       </c>
       <c r="D135" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E135" s="5"/>
       <c r="F135" s="4"/>
@@ -3186,14 +3186,14 @@
     </row>
     <row r="136" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A136" s="14" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B136" s="14"/>
       <c r="C136" s="14">
         <v>983210717</v>
       </c>
       <c r="D136" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E136" s="5"/>
       <c r="F136" s="4"/>
@@ -3202,14 +3202,14 @@
     </row>
     <row r="137" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A137" s="14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B137" s="14"/>
       <c r="C137" s="14">
         <v>935741979</v>
       </c>
       <c r="D137" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E137" s="5"/>
       <c r="F137" s="4"/>
@@ -3218,14 +3218,14 @@
     </row>
     <row r="138" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" s="14" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B138" s="14"/>
       <c r="C138" s="14">
         <v>954902084</v>
       </c>
       <c r="D138" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E138" s="5"/>
       <c r="F138" s="4"/>
@@ -3234,14 +3234,14 @@
     </row>
     <row r="139" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A139" s="14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B139" s="14"/>
       <c r="C139" s="14">
         <v>900049853</v>
       </c>
       <c r="D139" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E139" s="5"/>
       <c r="F139" s="4"/>
@@ -3250,14 +3250,14 @@
     </row>
     <row r="140" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A140" s="14" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B140" s="14"/>
       <c r="C140" s="14">
         <v>900049854</v>
       </c>
       <c r="D140" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E140" s="5"/>
       <c r="F140" s="4"/>
@@ -3266,14 +3266,14 @@
     </row>
     <row r="141" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A141" s="14" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B141" s="14"/>
       <c r="C141" s="14">
         <v>900049855</v>
       </c>
       <c r="D141" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E141" s="5"/>
       <c r="F141" s="4"/>
@@ -3282,14 +3282,14 @@
     </row>
     <row r="142" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" s="14" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B142" s="14"/>
       <c r="C142" s="14">
         <v>900049856</v>
       </c>
       <c r="D142" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E142" s="5"/>
       <c r="F142" s="4"/>
@@ -3298,14 +3298,14 @@
     </row>
     <row r="143" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A143" s="14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B143" s="14"/>
       <c r="C143" s="14">
         <v>900049857</v>
       </c>
       <c r="D143" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E143" s="5"/>
       <c r="F143" s="4"/>
@@ -3314,14 +3314,14 @@
     </row>
     <row r="144" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A144" s="14" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B144" s="14"/>
       <c r="C144" s="14">
         <v>900049858</v>
       </c>
       <c r="D144" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E144" s="5"/>
       <c r="F144" s="4"/>
@@ -3330,14 +3330,14 @@
     </row>
     <row r="145" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A145" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B145" s="14"/>
       <c r="C145" s="14">
         <v>900049859</v>
       </c>
       <c r="D145" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E145" s="5"/>
       <c r="F145" s="4"/>
@@ -3346,14 +3346,14 @@
     </row>
     <row r="146" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A146" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B146" s="14"/>
       <c r="C146" s="14">
         <v>900049860</v>
       </c>
       <c r="D146" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E146" s="5"/>
       <c r="F146" s="4"/>
@@ -3362,14 +3362,14 @@
     </row>
     <row r="147" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A147" s="14" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B147" s="14"/>
       <c r="C147" s="14">
         <v>900049861</v>
       </c>
       <c r="D147" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E147" s="5"/>
       <c r="F147" s="4"/>
@@ -3378,14 +3378,14 @@
     </row>
     <row r="148" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A148" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B148" s="14"/>
       <c r="C148" s="14">
         <v>900049862</v>
       </c>
       <c r="D148" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E148" s="5"/>
       <c r="F148" s="4"/>
@@ -3394,14 +3394,14 @@
     </row>
     <row r="149" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A149" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B149" s="14"/>
       <c r="C149" s="14">
         <v>900049863</v>
       </c>
       <c r="D149" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E149" s="5"/>
       <c r="F149" s="4"/>
@@ -3410,14 +3410,14 @@
     </row>
     <row r="150" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" s="14" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B150" s="14"/>
       <c r="C150" s="14">
         <v>900049864</v>
       </c>
       <c r="D150" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E150" s="5"/>
       <c r="F150" s="4"/>
@@ -3426,14 +3426,14 @@
     </row>
     <row r="151" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A151" s="14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B151" s="14"/>
       <c r="C151" s="14">
         <v>900049865</v>
       </c>
       <c r="D151" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E151" s="5"/>
       <c r="F151" s="4"/>
@@ -3442,14 +3442,14 @@
     </row>
     <row r="152" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A152" s="14" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B152" s="14"/>
       <c r="C152" s="14">
         <v>900049866</v>
       </c>
       <c r="D152" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E152" s="5"/>
       <c r="F152" s="4"/>
@@ -3458,14 +3458,14 @@
     </row>
     <row r="153" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A153" s="14" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B153" s="14"/>
       <c r="C153" s="14">
         <v>900049867</v>
       </c>
       <c r="D153" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E153" s="5"/>
       <c r="F153" s="4"/>
@@ -3474,14 +3474,14 @@
     </row>
     <row r="154" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A154" s="14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B154" s="14"/>
       <c r="C154" s="14">
         <v>946592840</v>
       </c>
       <c r="D154" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E154" s="5"/>
       <c r="F154" s="4"/>
@@ -3490,14 +3490,14 @@
     </row>
     <row r="155" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A155" s="14" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B155" s="14"/>
       <c r="C155" s="14">
         <v>977467731</v>
       </c>
       <c r="D155" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E155" s="5"/>
       <c r="F155" s="4"/>
@@ -3506,14 +3506,14 @@
     </row>
     <row r="156" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A156" s="14" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B156" s="14"/>
       <c r="C156" s="14">
         <v>964767294</v>
       </c>
       <c r="D156" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E156" s="5"/>
       <c r="F156" s="4"/>
@@ -3522,14 +3522,14 @@
     </row>
     <row r="157" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A157" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B157" s="14"/>
       <c r="C157" s="14">
         <v>935741979</v>
       </c>
       <c r="D157" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E157" s="5"/>
       <c r="F157" s="4"/>
@@ -3538,14 +3538,14 @@
     </row>
     <row r="158" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A158" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B158" s="14"/>
       <c r="C158" s="14">
         <v>991495906</v>
       </c>
       <c r="D158" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E158" s="5"/>
       <c r="F158" s="4"/>
@@ -3554,14 +3554,14 @@
     </row>
     <row r="159" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A159" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B159" s="14"/>
       <c r="C159" s="14">
         <v>946784628</v>
       </c>
       <c r="D159" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E159" s="5"/>
       <c r="F159" s="4"/>
@@ -3570,14 +3570,14 @@
     </row>
     <row r="160" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A160" s="14" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B160" s="14"/>
       <c r="C160" s="14">
         <v>947366117</v>
       </c>
       <c r="D160" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E160" s="5"/>
       <c r="F160" s="4"/>
@@ -3586,14 +3586,14 @@
     </row>
     <row r="161" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A161" s="14" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B161" s="14"/>
       <c r="C161" s="14">
         <v>954243859</v>
       </c>
       <c r="D161" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E161" s="5"/>
       <c r="F161" s="4"/>
@@ -3602,14 +3602,14 @@
     </row>
     <row r="162" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A162" s="14" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B162" s="14"/>
       <c r="C162" s="14">
         <v>923269037</v>
       </c>
       <c r="D162" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E162" s="5"/>
       <c r="F162" s="4"/>
@@ -3618,14 +3618,14 @@
     </row>
     <row r="163" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A163" s="14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B163" s="14"/>
       <c r="C163" s="14">
         <v>984565061</v>
       </c>
       <c r="D163" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E163" s="5"/>
       <c r="F163" s="4"/>
@@ -3634,14 +3634,14 @@
     </row>
     <row r="164" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A164" s="14" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B164" s="14"/>
       <c r="C164" s="14">
         <v>919729393</v>
       </c>
       <c r="D164" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E164" s="5"/>
       <c r="F164" s="4"/>
@@ -3650,12 +3650,12 @@
     </row>
     <row r="165" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A165" s="14" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B165" s="14"/>
       <c r="C165" s="14"/>
       <c r="D165" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E165" s="5"/>
       <c r="F165" s="4"/>
@@ -3664,12 +3664,12 @@
     </row>
     <row r="166" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A166" s="14" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B166" s="14"/>
       <c r="C166" s="14"/>
       <c r="D166" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E166" s="5"/>
       <c r="F166" s="4"/>
@@ -3678,12 +3678,12 @@
     </row>
     <row r="167" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A167" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B167" s="14"/>
       <c r="C167" s="14"/>
       <c r="D167" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E167" s="5"/>
       <c r="F167" s="4"/>

</xml_diff>